<commit_message>
feat: working +- another template
</commit_message>
<xml_diff>
--- a/ids.xlsx
+++ b/ids.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30210"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{98AAC513-C45E-4AF2-81F9-316A22C97B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D11197C0-9264-4892-ABA6-F31B5F8FF1F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -63,6 +63,14 @@
       <color rgb="FF104861"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -91,11 +99,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -410,40 +419,66 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:3">
       <c r="A2" s="2">
         <v>8000066095</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:3">
       <c r="A3" s="3">
         <v>8000066149</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:3">
       <c r="A4" s="2">
         <v>8000066206</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:3">
       <c r="A5" s="3">
         <v>8000066329</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:3">
       <c r="A6" s="2">
         <v>8000066397</v>
+      </c>
+      <c r="C6" s="4"/>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="3">
+        <v>8000066422</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="2">
+        <v>8000066604</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="3">
+        <v>8000066644</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="2">
+        <v>8000066696</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="3">
+        <v>8000066776</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: reading some pdf images
</commit_message>
<xml_diff>
--- a/ids.xlsx
+++ b/ids.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30210"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D11197C0-9264-4892-ABA6-F31B5F8FF1F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CAAE826E-99B2-4BCB-92F2-CE263461E5A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -102,9 +102,9 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -419,7 +419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -431,54 +431,154 @@
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>8000066095</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="3">
+      <c r="A3" s="4">
         <v>8000066149</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="2">
+      <c r="A4" s="3">
         <v>8000066206</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="3">
+      <c r="A5" s="4">
         <v>8000066329</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="2">
+      <c r="A6" s="3">
         <v>8000066397</v>
       </c>
-      <c r="C6" s="4"/>
+      <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="3">
+      <c r="A7" s="4">
         <v>8000066422</v>
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="2">
+      <c r="A8" s="3">
         <v>8000066604</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" s="3">
+      <c r="A9" s="4">
         <v>8000066644</v>
       </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" s="2">
+      <c r="A10" s="3">
         <v>8000066696</v>
       </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" s="3">
+      <c r="A11" s="4">
         <v>8000066776</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="3">
+        <v>8000066812</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="4">
+        <v>8000066866</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="3">
+        <v>8000066922</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="4">
+        <v>8000066987</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="3">
+        <v>8000067078</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="4">
+        <v>8000067135</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="3">
+        <v>8000067287</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="4">
+        <v>8000067308</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="3">
+        <v>8000067329</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" s="4">
+        <v>8000067346</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" s="3">
+        <v>8000067408</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" s="4">
+        <v>8000067426</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" s="3">
+        <v>8000067486</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" s="4">
+        <v>8000067563</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" s="3">
+        <v>8000067568</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" s="4">
+        <v>8000067569</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" s="3">
+        <v>8000067597</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" s="4">
+        <v>8000067608</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30" s="3">
+        <v>8000067617</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" s="4">
+        <v>8000067623</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: increased accuracy of ocr
</commit_message>
<xml_diff>
--- a/ids.xlsx
+++ b/ids.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30210"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7C9FC3EC-CA5F-4FB8-9261-D200A1FF35E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADD12B94-929F-49B9-86FB-8DB39F1DD89B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -419,7 +419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -432,277 +432,527 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="3">
-        <v>8000068556</v>
+        <v>8000066095</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="4">
-        <v>8000068579</v>
+        <v>8000066149</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="3">
-        <v>8000068615</v>
+        <v>8000066206</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="4">
-        <v>8000068649</v>
+        <v>8000066329</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="3">
-        <v>8000068699</v>
+        <v>8000066397</v>
       </c>
       <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="4">
-        <v>8000068719</v>
+        <v>8000066422</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="3">
-        <v>8000068797</v>
+        <v>8000066604</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="4">
-        <v>8000068805</v>
+        <v>8000066644</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="3">
-        <v>8000068838</v>
+        <v>8000066696</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="4">
-        <v>8000068944</v>
+        <v>8000066776</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="3">
-        <v>8000068951</v>
+        <v>8000066812</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="4">
-        <v>8000069046</v>
+        <v>8000066866</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="3">
-        <v>8000069095</v>
+        <v>8000066922</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="4">
-        <v>8000069105</v>
+        <v>8000066987</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="3">
-        <v>8000069193</v>
+        <v>8000067078</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="4">
-        <v>8000069256</v>
+        <v>8000067135</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="3">
-        <v>8000069337</v>
+        <v>8000067287</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="4">
-        <v>8000069459</v>
+        <v>8000067308</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="3">
-        <v>8000069468</v>
+        <v>8000067329</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="4">
-        <v>8000069581</v>
+        <v>8000067346</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" s="3">
-        <v>8000069598</v>
+        <v>8000067408</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" s="4">
-        <v>8000069641</v>
+        <v>8000067426</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" s="3">
-        <v>8000070038</v>
+        <v>8000067486</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" s="4">
-        <v>8000070139</v>
+        <v>8000067563</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" s="3">
-        <v>8000070167</v>
+        <v>8000067568</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" s="4">
-        <v>8000070193</v>
+        <v>8000067569</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" s="3">
-        <v>8000070370</v>
+        <v>8000067597</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" s="4">
-        <v>8000070412</v>
+        <v>8000067608</v>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" s="3">
-        <v>8000070512</v>
+        <v>8000067617</v>
       </c>
     </row>
     <row r="31" spans="1:1">
       <c r="A31" s="4">
-        <v>8000070570</v>
+        <v>8000067623</v>
       </c>
     </row>
     <row r="32" spans="1:1">
       <c r="A32" s="3">
-        <v>8000070578</v>
+        <v>8000067694</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" s="4">
-        <v>8000070599</v>
+        <v>8000067712</v>
       </c>
     </row>
     <row r="34" spans="1:1">
       <c r="A34" s="3">
-        <v>8000070611</v>
+        <v>8000067727</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" s="4">
-        <v>8000070747</v>
+        <v>8000067746</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" s="3">
-        <v>8000070757</v>
+        <v>8000067752</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" s="4">
-        <v>8000070811</v>
+        <v>8000067817</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" s="3">
-        <v>8000071026</v>
+        <v>8000067862</v>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" s="4">
-        <v>8000071105</v>
+        <v>8000067890</v>
       </c>
     </row>
     <row r="40" spans="1:1">
       <c r="A40" s="3">
-        <v>8000071161</v>
+        <v>8000067922</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" s="4">
-        <v>8000071267</v>
+        <v>8000067933</v>
       </c>
     </row>
     <row r="42" spans="1:1">
       <c r="A42" s="3">
-        <v>8000071296</v>
+        <v>8000067937</v>
       </c>
     </row>
     <row r="43" spans="1:1">
       <c r="A43" s="4">
-        <v>8000071544</v>
+        <v>8000067958</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" s="3">
-        <v>8000071559</v>
+        <v>8000068014</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" s="4">
-        <v>8000071609</v>
+        <v>8000068121</v>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" s="3">
-        <v>8000071766</v>
+        <v>8000068129</v>
       </c>
     </row>
     <row r="47" spans="1:1">
       <c r="A47" s="4">
-        <v>8000071825</v>
+        <v>8000068191</v>
       </c>
     </row>
     <row r="48" spans="1:1">
       <c r="A48" s="3">
-        <v>8000071999</v>
+        <v>8000068257</v>
       </c>
     </row>
     <row r="49" spans="1:1">
       <c r="A49" s="4">
-        <v>8000072005</v>
+        <v>8000068352</v>
       </c>
     </row>
     <row r="50" spans="1:1">
       <c r="A50" s="3">
-        <v>8000072055</v>
+        <v>8000068428</v>
       </c>
     </row>
     <row r="51" spans="1:1">
       <c r="A51" s="4">
-        <v>8000072259</v>
+        <v>8000068487</v>
       </c>
     </row>
     <row r="52" spans="1:1">
       <c r="A52" s="3">
-        <v>8000072354</v>
+        <v>8000068556</v>
       </c>
     </row>
     <row r="53" spans="1:1">
       <c r="A53" s="4">
-        <v>8000072696</v>
+        <v>8000068579</v>
       </c>
     </row>
     <row r="54" spans="1:1">
       <c r="A54" s="3">
-        <v>8000072892</v>
+        <v>8000068615</v>
       </c>
     </row>
     <row r="55" spans="1:1">
       <c r="A55" s="4">
-        <v>8000073428</v>
+        <v>8000068649</v>
       </c>
     </row>
     <row r="56" spans="1:1">
       <c r="A56" s="3">
+        <v>8000068699</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57" s="4">
+        <v>8000068719</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58" s="3">
+        <v>8000068797</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59" s="4">
+        <v>8000068805</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60" s="3">
+        <v>8000068838</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" s="4">
+        <v>8000068944</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62" s="3">
+        <v>8000068951</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" s="4">
+        <v>8000069046</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1">
+      <c r="A64" s="3">
+        <v>8000069095</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" s="4">
+        <v>8000069105</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" s="3">
+        <v>8000069193</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67" s="4">
+        <v>8000069256</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" s="3">
+        <v>8000069337</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69" s="4">
+        <v>8000069459</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70" s="3">
+        <v>8000069468</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71" s="4">
+        <v>8000069581</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" s="3">
+        <v>8000069598</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73" s="4">
+        <v>8000069641</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74" s="3">
+        <v>8000070038</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" s="4">
+        <v>8000070139</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76" s="3">
+        <v>8000070167</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77" s="4">
+        <v>8000070193</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1">
+      <c r="A78" s="3">
+        <v>8000070370</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79" s="4">
+        <v>8000070412</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1">
+      <c r="A80" s="3">
+        <v>8000070512</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81" s="4">
+        <v>8000070570</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1">
+      <c r="A82" s="3">
+        <v>8000070578</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83" s="4">
+        <v>8000070599</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84" s="3">
+        <v>8000070611</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1">
+      <c r="A85" s="4">
+        <v>8000070747</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1">
+      <c r="A86" s="3">
+        <v>8000070757</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1">
+      <c r="A87" s="4">
+        <v>8000070811</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1">
+      <c r="A88" s="3">
+        <v>8000071026</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1">
+      <c r="A89" s="4">
+        <v>8000071105</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1">
+      <c r="A90" s="3">
+        <v>8000071161</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1">
+      <c r="A91" s="4">
+        <v>8000071267</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1">
+      <c r="A92" s="3">
+        <v>8000071296</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1">
+      <c r="A93" s="4">
+        <v>8000071544</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1">
+      <c r="A94" s="3">
+        <v>8000071559</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95" s="4">
+        <v>8000071609</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1">
+      <c r="A96" s="3">
+        <v>8000071766</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97" s="4">
+        <v>8000071825</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1">
+      <c r="A98" s="3">
+        <v>8000071999</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99" s="4">
+        <v>8000072005</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1">
+      <c r="A100" s="3">
+        <v>8000072055</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1">
+      <c r="A101" s="4">
+        <v>8000072259</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1">
+      <c r="A102" s="3">
+        <v>8000072354</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103" s="4">
+        <v>8000072696</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1">
+      <c r="A104" s="3">
+        <v>8000072892</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" s="4">
+        <v>8000073428</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1">
+      <c r="A106" s="3">
         <v>8000073747</v>
       </c>
     </row>

</xml_diff>